<commit_message>
Some adjustments to Cashflow graph in Excel template.
</commit_message>
<xml_diff>
--- a/financeTemplate.xlsx
+++ b/financeTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbyrne/Dropbox/eclipse-workspace/finance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA555E7-4C94-8B43-A00E-D16939F65569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FF4084-65EC-8942-9F66-2FC5E5568893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42040" yWindow="2340" windowWidth="67820" windowHeight="28940" activeTab="1" xr2:uid="{535C330D-3385-BC47-B3AB-34923AEE4912}"/>
+    <workbookView xWindow="39800" yWindow="1640" windowWidth="67820" windowHeight="28940" activeTab="3" xr2:uid="{535C330D-3385-BC47-B3AB-34923AEE4912}"/>
   </bookViews>
   <sheets>
     <sheet name="output (2)" sheetId="21" r:id="rId1"/>
@@ -1411,9 +1411,6 @@
     <t>TD AUTO FINANCE WEB PAY   250426|-441.880004882813</t>
   </si>
   <si>
-    <t>amount over/under linear prediction</t>
-  </si>
-  <si>
     <t>If I stopped spending totally at this point, would I be within budget
 considering future TXs?  I would have spent this much considering
 future TXs:</t>
@@ -1660,6 +1657,9 @@
   </si>
   <si>
     <t>Income Cumulative</t>
+  </si>
+  <si>
+    <t>amount -over/+under linear prediction</t>
   </si>
 </sst>
 </file>
@@ -9963,7 +9963,7 @@
         <v>45803</v>
       </c>
       <c r="B22" s="41" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C22">
         <v>-81.980003356933594</v>
@@ -10193,7 +10193,7 @@
         <v>45804</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C32">
         <v>-22.090000152587891</v>
@@ -10216,7 +10216,7 @@
         <v>45804</v>
       </c>
       <c r="B33" s="41" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C33">
         <v>-5.9200000762939453</v>
@@ -10285,7 +10285,7 @@
         <v>45805</v>
       </c>
       <c r="B36" s="41" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C36">
         <v>-42.830001831054688</v>
@@ -10308,7 +10308,7 @@
         <v>45805</v>
       </c>
       <c r="B37" s="41" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C37">
         <v>-24.629999160766602</v>
@@ -10469,7 +10469,7 @@
         <v>45805</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C44">
         <v>-515</v>
@@ -10492,7 +10492,7 @@
         <v>45805</v>
       </c>
       <c r="B45" s="41" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C45">
         <v>-73.330001831054688</v>
@@ -10515,7 +10515,7 @@
         <v>45805</v>
       </c>
       <c r="B46" s="41" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C46">
         <v>-441.8800048828125</v>
@@ -10561,7 +10561,7 @@
         <v>45806</v>
       </c>
       <c r="B48" s="41" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C48">
         <v>-14.989999771118164</v>
@@ -10584,7 +10584,7 @@
         <v>45806</v>
       </c>
       <c r="B49" s="41" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C49">
         <v>15.159999847412109</v>
@@ -10630,7 +10630,7 @@
         <v>45807</v>
       </c>
       <c r="B51" s="41" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C51">
         <v>-16.479999542236328</v>
@@ -10699,7 +10699,7 @@
         <v>45810</v>
       </c>
       <c r="B54" s="41" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C54">
         <v>3.5</v>
@@ -10722,7 +10722,7 @@
         <v>45810</v>
       </c>
       <c r="B55" s="41" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C55">
         <v>-2.3599998950958252</v>
@@ -10745,7 +10745,7 @@
         <v>45810</v>
       </c>
       <c r="B56" s="41" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C56">
         <v>-5.0999999046325684</v>
@@ -10768,7 +10768,7 @@
         <v>45810</v>
       </c>
       <c r="B57" s="41" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C57">
         <v>-3.1500000953674316</v>
@@ -10791,7 +10791,7 @@
         <v>45810</v>
       </c>
       <c r="B58" s="41" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C58">
         <v>-74.790000915527344</v>
@@ -10814,7 +10814,7 @@
         <v>45810</v>
       </c>
       <c r="B59" s="41" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C59">
         <v>-59.090000152587891</v>
@@ -10837,7 +10837,7 @@
         <v>45811</v>
       </c>
       <c r="B60" s="41" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C60">
         <v>-5.5900001525878906</v>
@@ -10860,7 +10860,7 @@
         <v>45811</v>
       </c>
       <c r="B61" s="41" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C61">
         <v>-13.920000076293945</v>
@@ -10883,7 +10883,7 @@
         <v>45811</v>
       </c>
       <c r="B62" s="41" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C62">
         <v>-359.22000122070312</v>
@@ -10975,7 +10975,7 @@
         <v>45813</v>
       </c>
       <c r="B66" s="41" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C66">
         <v>-3.0899999141693115</v>
@@ -11090,7 +11090,7 @@
         <v>45815</v>
       </c>
       <c r="B71" s="41" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C71">
         <v>-12</v>
@@ -11113,7 +11113,7 @@
         <v>45815</v>
       </c>
       <c r="B72" s="41" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C72">
         <v>-10</v>
@@ -11136,7 +11136,7 @@
         <v>45815</v>
       </c>
       <c r="B73" s="41" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C73">
         <v>-5</v>
@@ -11159,7 +11159,7 @@
         <v>45815</v>
       </c>
       <c r="B74" s="41" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C74">
         <v>-205.47999572753906</v>
@@ -11182,7 +11182,7 @@
         <v>45816</v>
       </c>
       <c r="B75" s="41" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C75">
         <v>-20.030000686645508</v>
@@ -11205,7 +11205,7 @@
         <v>45816</v>
       </c>
       <c r="B76" s="41" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C76">
         <v>-5</v>
@@ -11251,7 +11251,7 @@
         <v>45817</v>
       </c>
       <c r="B78" s="41" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C78">
         <v>-3.2400000095367432</v>
@@ -11274,7 +11274,7 @@
         <v>45817</v>
       </c>
       <c r="B79" s="41" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C79">
         <v>-300</v>
@@ -11297,7 +11297,7 @@
         <v>45817</v>
       </c>
       <c r="B80" s="41" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C80">
         <v>-474.6400146484375</v>
@@ -11343,7 +11343,7 @@
         <v>45818</v>
       </c>
       <c r="B82" s="41" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C82">
         <v>-14.979999542236328</v>
@@ -11366,7 +11366,7 @@
         <v>45818</v>
       </c>
       <c r="B83" s="41" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C83">
         <v>-441.8800048828125</v>
@@ -11435,7 +11435,7 @@
         <v>45820</v>
       </c>
       <c r="B86" s="41" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C86">
         <v>-1182.3599853515625</v>
@@ -11458,7 +11458,7 @@
         <v>45820</v>
       </c>
       <c r="B87" s="41" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C87">
         <v>2877.22998046875</v>
@@ -11481,7 +11481,7 @@
         <v>45821</v>
       </c>
       <c r="B88" s="41" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C88">
         <v>-12.5</v>
@@ -11504,7 +11504,7 @@
         <v>45821</v>
       </c>
       <c r="B89" s="41" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C89">
         <v>-77.720001220703125</v>
@@ -11527,7 +11527,7 @@
         <v>45821</v>
       </c>
       <c r="B90" s="41" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C90">
         <v>-2.9900000095367432</v>
@@ -11550,13 +11550,13 @@
         <v>45822</v>
       </c>
       <c r="B91" s="41" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C91">
         <v>-27</v>
       </c>
       <c r="D91" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E91" s="41" t="s">
         <v>174</v>
@@ -11854,7 +11854,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B18">
         <v>-27</v>
@@ -31375,7 +31375,7 @@
         <v>48</v>
       </c>
       <c r="W1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>12</v>
@@ -33047,7 +33047,7 @@
         <v>45803</v>
       </c>
       <c r="B22" s="48" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C22" s="44">
         <v>-81.980003356933594</v>
@@ -33847,7 +33847,7 @@
         <v>45804</v>
       </c>
       <c r="B32" s="48" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C32" s="44">
         <v>-22.090000152587891</v>
@@ -33927,7 +33927,7 @@
         <v>45804</v>
       </c>
       <c r="B33" s="51" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C33" s="45">
         <v>-5.9200000762939453</v>
@@ -34167,7 +34167,7 @@
         <v>45805</v>
       </c>
       <c r="B36" s="48" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C36" s="44">
         <v>-42.830001831054688</v>
@@ -34247,7 +34247,7 @@
         <v>45805</v>
       </c>
       <c r="B37" s="51" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C37" s="45">
         <v>-24.629999160766602</v>
@@ -34836,7 +34836,7 @@
         <v>45805</v>
       </c>
       <c r="B44" s="48" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C44" s="44">
         <v>-515</v>
@@ -34916,7 +34916,7 @@
         <v>45805</v>
       </c>
       <c r="B45" s="51" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C45" s="45">
         <v>-73.330001831054688</v>
@@ -34996,7 +34996,7 @@
         <v>45805</v>
       </c>
       <c r="B46" s="48" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C46" s="44">
         <v>-441.8800048828125</v>
@@ -35156,7 +35156,7 @@
         <v>45806</v>
       </c>
       <c r="B48" s="48" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C48" s="44">
         <v>-14.989999771118164</v>
@@ -35236,7 +35236,7 @@
         <v>45806</v>
       </c>
       <c r="B49" s="51" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C49" s="45">
         <v>15.159999847412109</v>
@@ -35396,7 +35396,7 @@
         <v>45807</v>
       </c>
       <c r="B51" s="51" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C51" s="45">
         <v>-16.479999542236328</v>
@@ -35636,7 +35636,7 @@
         <v>45810</v>
       </c>
       <c r="B54" s="48" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C54" s="44">
         <v>3.5</v>
@@ -35716,7 +35716,7 @@
         <v>45810</v>
       </c>
       <c r="B55" s="51" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C55" s="45">
         <v>-2.3599998950958252</v>
@@ -35796,7 +35796,7 @@
         <v>45810</v>
       </c>
       <c r="B56" s="48" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C56" s="44">
         <v>-5.0999999046325684</v>
@@ -35876,7 +35876,7 @@
         <v>45810</v>
       </c>
       <c r="B57" s="51" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C57" s="45">
         <v>-3.1500000953674316</v>
@@ -35956,7 +35956,7 @@
         <v>45810</v>
       </c>
       <c r="B58" s="48" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C58" s="44">
         <v>-74.790000915527344</v>
@@ -36036,7 +36036,7 @@
         <v>45810</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C59" s="45">
         <v>-59.090000152587891</v>
@@ -36116,7 +36116,7 @@
         <v>45811</v>
       </c>
       <c r="B60" s="48" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C60" s="44">
         <v>-5.5900001525878906</v>
@@ -36196,7 +36196,7 @@
         <v>45811</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C61" s="45">
         <v>-13.920000076293945</v>
@@ -36276,7 +36276,7 @@
         <v>45811</v>
       </c>
       <c r="B62" s="48" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C62" s="44">
         <v>-359.22000122070312</v>
@@ -36596,7 +36596,7 @@
         <v>45813</v>
       </c>
       <c r="B66" s="48" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C66" s="44">
         <v>-3.0899999141693115</v>
@@ -36996,7 +36996,7 @@
         <v>45815</v>
       </c>
       <c r="B71" s="51" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C71" s="45">
         <v>-12</v>
@@ -37076,7 +37076,7 @@
         <v>45815</v>
       </c>
       <c r="B72" s="48" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C72" s="44">
         <v>-10</v>
@@ -37156,7 +37156,7 @@
         <v>45815</v>
       </c>
       <c r="B73" s="51" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C73" s="45">
         <v>-5</v>
@@ -37236,7 +37236,7 @@
         <v>45815</v>
       </c>
       <c r="B74" s="48" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C74" s="44">
         <v>-205.47999572753906</v>
@@ -37316,7 +37316,7 @@
         <v>45816</v>
       </c>
       <c r="B75" s="51" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C75" s="45">
         <v>-20.030000686645508</v>
@@ -37396,7 +37396,7 @@
         <v>45816</v>
       </c>
       <c r="B76" s="48" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C76" s="44">
         <v>-5</v>
@@ -37556,7 +37556,7 @@
         <v>45817</v>
       </c>
       <c r="B78" s="48" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C78" s="44">
         <v>-3.2400000095367432</v>
@@ -37636,7 +37636,7 @@
         <v>45817</v>
       </c>
       <c r="B79" s="51" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C79" s="45">
         <v>-300</v>
@@ -37716,7 +37716,7 @@
         <v>45817</v>
       </c>
       <c r="B80" s="48" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C80" s="44">
         <v>-474.6400146484375</v>
@@ -37876,7 +37876,7 @@
         <v>45818</v>
       </c>
       <c r="B82" s="48" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C82" s="44">
         <v>-14.979999542236328</v>
@@ -37956,7 +37956,7 @@
         <v>45818</v>
       </c>
       <c r="B83" s="51" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C83" s="45">
         <v>-441.8800048828125</v>
@@ -38196,7 +38196,7 @@
         <v>45820</v>
       </c>
       <c r="B86" s="48" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C86" s="44">
         <v>-1182.3599853515625</v>
@@ -38276,7 +38276,7 @@
         <v>45820</v>
       </c>
       <c r="B87" s="51" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C87" s="45">
         <v>2877.22998046875</v>
@@ -38356,7 +38356,7 @@
         <v>45821</v>
       </c>
       <c r="B88" s="48" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C88" s="44">
         <v>-12.5</v>
@@ -38436,7 +38436,7 @@
         <v>45821</v>
       </c>
       <c r="B89" s="51" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C89" s="45">
         <v>-77.720001220703125</v>
@@ -38516,7 +38516,7 @@
         <v>45821</v>
       </c>
       <c r="B90" s="48" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C90" s="44">
         <v>-2.9900000095367432</v>
@@ -38596,13 +38596,13 @@
         <v>45822</v>
       </c>
       <c r="B91" s="51" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C91" s="45">
         <v>-27</v>
       </c>
       <c r="D91" s="51" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E91" s="51" t="s">
         <v>174</v>
@@ -47819,10 +47819,10 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B29" s="41" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -47875,7 +47875,7 @@
         <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D2" s="1">
         <v>-449.6400146484375</v>
@@ -47911,7 +47911,7 @@
         <v>13.84</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D4" s="1">
         <v>-345.38000122070315</v>
@@ -47929,7 +47929,7 @@
         <v>302.95</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D5" s="1">
         <v>2.9499999999999886</v>
@@ -47947,7 +47947,7 @@
         <v>518.29999999999995</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D6" s="1">
         <v>219.8599975585937</v>
@@ -47971,7 +47971,7 @@
         <v>1071.28</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D7" s="1">
         <v>920.33999755859372</v>
@@ -47996,7 +47996,7 @@
         <v>87.9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D8" s="1">
         <v>6.4100021362304744</v>
@@ -48020,7 +48020,7 @@
         <v>69.349999999999994</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D9" s="1">
         <v>-5.4400009155273494</v>
@@ -48045,7 +48045,7 @@
         <v>76.650000000000006</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D10" s="1">
         <v>17.559999847412115</v>
@@ -48108,7 +48108,7 @@
         <v>40</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D13" s="1">
         <v>2.8300018310546875</v>
@@ -48123,13 +48123,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B14">
         <v>30</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D14" s="1">
         <v>3</v>
@@ -48150,7 +48150,7 @@
         <v>19.16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D15" s="1">
         <v>13.56999984741211</v>
@@ -48168,7 +48168,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D16" s="1">
         <v>-2.3599998950958252</v>
@@ -48189,7 +48189,7 @@
         <v>40</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D17" s="1">
         <v>36.5</v>
@@ -48211,7 +48211,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>351</v>
+        <v>433</v>
       </c>
       <c r="J18" t="s">
         <v>333</v>
@@ -48499,7 +48499,7 @@
       </c>
       <c r="E31" s="1"/>
       <c r="G31" s="40" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H31" s="4">
         <f>J12+ABS(H29)</f>
@@ -48522,7 +48522,7 @@
     </row>
     <row r="33" spans="7:11" x14ac:dyDescent="0.2">
       <c r="G33" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H33">
         <f>J9-H31</f>
@@ -48545,7 +48545,7 @@
     </row>
     <row r="35" spans="7:11" x14ac:dyDescent="0.2">
       <c r="G35" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="J35">
         <v>20</v>
@@ -48556,7 +48556,7 @@
     </row>
     <row r="36" spans="7:11" x14ac:dyDescent="0.2">
       <c r="G36" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="H36">
         <v>81.98</v>
@@ -48570,7 +48570,7 @@
     </row>
     <row r="37" spans="7:11" x14ac:dyDescent="0.2">
       <c r="G37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="H37">
         <v>154.94</v>
@@ -48584,7 +48584,7 @@
     </row>
     <row r="38" spans="7:11" x14ac:dyDescent="0.2">
       <c r="G38" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H38">
         <v>42.83</v>
@@ -48641,7 +48641,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="48" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B1">
         <v>474.64</v>
@@ -48657,7 +48657,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B3">
         <v>359.22</v>
@@ -48665,7 +48665,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="51" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B4">
         <v>300</v>
@@ -48673,7 +48673,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="48" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B5">
         <v>298.44</v>
@@ -48681,7 +48681,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="51" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B6">
         <v>150.94</v>
@@ -48689,7 +48689,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="48" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B7">
         <v>81.489999999999995</v>
@@ -48697,7 +48697,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="51" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B8">
         <v>74.790000000000006</v>
@@ -48705,7 +48705,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="48" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B9">
         <v>59.09</v>
@@ -48729,7 +48729,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="51" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B12">
         <v>37.17</v>
@@ -48737,7 +48737,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="48" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B13">
         <v>27</v>
@@ -48745,7 +48745,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="51" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B14">
         <v>5.59</v>
@@ -48753,7 +48753,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="48" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B15">
         <v>2.36</v>
@@ -49904,10 +49904,10 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B22" s="41" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -50881,7 +50881,7 @@
         <v>35.22</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I2" t="b">
         <f t="shared" ref="I2:I26" si="1">ISBLANK(G2)</f>
@@ -50920,7 +50920,7 @@
         <v>9.9600000000000009</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I3" t="b">
         <f t="shared" si="1"/>
@@ -50959,7 +50959,7 @@
         <v>17.04</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I4" t="b">
         <f t="shared" si="1"/>
@@ -50998,7 +50998,7 @@
         <v>29.06</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I5" t="b">
         <f t="shared" si="1"/>
@@ -51037,7 +51037,7 @@
         <v>21.74</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I6" t="b">
         <f t="shared" si="1"/>
@@ -51076,7 +51076,7 @@
         <v>0.82</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I7" t="b">
         <f t="shared" si="1"/>
@@ -51193,7 +51193,7 @@
         <v>2.89</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I10" t="b">
         <f t="shared" si="1"/>
@@ -51232,7 +51232,7 @@
         <v>0.72</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I11" t="b">
         <f t="shared" si="1"/>
@@ -51271,7 +51271,7 @@
         <v>6.08</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="I12" t="b">
         <f t="shared" si="1"/>
@@ -51310,7 +51310,7 @@
         <v>5.72</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I13" t="b">
         <f t="shared" si="1"/>
@@ -51349,7 +51349,7 @@
         <v>5.35</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I14" t="b">
         <f t="shared" si="1"/>
@@ -51388,7 +51388,7 @@
         <v>1.32</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="I15" t="b">
         <f t="shared" si="1"/>
@@ -51466,7 +51466,7 @@
         <v>0.46</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I17" t="b">
         <f t="shared" si="1"/>
@@ -51505,7 +51505,7 @@
         <v>2.2799999999999998</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I18" t="b">
         <f t="shared" si="1"/>
@@ -51544,7 +51544,7 @@
         <v>0.66</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I19" t="b">
         <f t="shared" si="1"/>
@@ -51583,7 +51583,7 @@
         <v>2.52</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="I20" t="b">
         <f t="shared" si="1"/>
@@ -51661,7 +51661,7 @@
         <v>1.32</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I22" t="b">
         <f t="shared" si="1"/>
@@ -51682,13 +51682,13 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="41" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B23">
         <v>-253.00999450683594</v>
       </c>
       <c r="C23" s="41" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -51799,13 +51799,13 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B26">
         <v>-123.20999908447266</v>
       </c>
       <c r="C26" s="41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D26">
         <v>163.35</v>
@@ -51817,7 +51817,7 @@
         <v>0.99</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I26" t="b">
         <f t="shared" si="1"/>
@@ -51856,7 +51856,7 @@
         <v>1.32</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I27" t="b">
         <f>ISBLANK(G33)</f>
@@ -51895,7 +51895,7 @@
         <v>0.63</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I28" t="b">
         <f>ISBLANK(G34)</f>
@@ -51957,7 +51957,7 @@
         <v>0.13</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
@@ -52008,13 +52008,13 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="41" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B33">
         <v>2595.800048828125</v>
       </c>
       <c r="C33" s="41" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D33">
         <v>0</v>

</xml_diff>